<commit_message>
Dashboard chart layout fixed: tables on top, spaced 2x2 chart grid below
The chart anchors overlapped (a 17-row-tall chart anchored 10 rows above
the next). Charts now sit in their own band under the tables — revenue
stream stack and cumulative-cash line side by side, milestones and
use-of-funds below — with helper chart data plainly labelled at the foot.
Verified: 0 formula failures, headline cells still tie to the model.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H812bzJCmkxEBTne82bnSQ
</commit_message>
<xml_diff>
--- a/GetLucky_Pro_Forma_v4.xlsx
+++ b/GetLucky_Pro_Forma_v4.xlsx
@@ -32,7 +32,7 @@
     <numFmt numFmtId="170" formatCode="$0.00"/>
     <numFmt numFmtId="171" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -191,6 +191,12 @@
       <color rgb="009A937B"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009A937B"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -241,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -325,6 +331,8 @@
     <xf numFmtId="167" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -608,7 +616,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Cumulative cash (ZAR) — peak drawdown inside the raise</a:t>
+              <a:t>Cumulative cash (ZAR) — trough inside the raise</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -707,9 +715,6 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
-              <a:srgbClr val="345230"/>
-            </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -749,12 +754,12 @@
           </dPt>
           <cat>
             <numRef>
-              <f>'Dashboard'!$O$48:$O$50</f>
+              <f>'Dashboard'!$B$95:$B$97</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$P$48:$P$50</f>
+              <f>'Dashboard'!$C$95:$C$97</f>
             </numRef>
           </val>
         </ser>
@@ -878,12 +883,12 @@
           </dPt>
           <cat>
             <numRef>
-              <f>'Dashboard'!$O$41:$O$45</f>
+              <f>'Dashboard'!$B$89:$B$93</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$P$41:$P$45</f>
+              <f>'Dashboard'!$C$89:$C$93</f>
             </numRef>
           </val>
         </ser>
@@ -891,7 +896,7 @@
       </pieChart>
     </plotArea>
     <legend>
-      <legendPos val="b"/>
+      <legendPos val="r"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -903,12 +908,12 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>40</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5580000" cy="3024000"/>
+    <ext cx="5400000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -925,12 +930,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>9</col>
       <colOff>0</colOff>
-      <row>21</row>
+      <row>40</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5580000" cy="3024000"/>
+    <ext cx="5400000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -947,12 +952,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>61</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3384000" cy="2736000"/>
+    <ext cx="5400000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -969,12 +974,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>11</col>
+      <col>9</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>61</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2376000" cy="2736000"/>
+    <ext cx="5400000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="4" name="Chart 4"/>
@@ -1497,24 +1502,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:P51"/>
+  <dimension ref="B2:H97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="4" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
-    <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1534,7 +1532,7 @@
     <row r="5">
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Revenue 2029</t>
+          <t>REVENUE 2029</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -1544,20 +1542,20 @@
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>Milestone Dec 2029</t>
+          <t>MILESTONE DEC 2029</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="55">
+      <c r="B6" s="77">
         <f>Annual!E17</f>
         <v/>
       </c>
-      <c r="D6" s="55">
+      <c r="D6" s="77">
         <f>Annual!E27</f>
         <v/>
       </c>
-      <c r="F6" s="55">
+      <c r="F6" s="77">
         <f>Valuation!D10</f>
         <v/>
       </c>
@@ -1565,17 +1563,17 @@
     <row r="8">
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>Investor multiple 2029</t>
+          <t>INVESTOR MULTIPLE 2029</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Peak drawdown</t>
+          <t>PEAK DRAWDOWN</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>Subscribers 2032</t>
+          <t>SUBSCRIBERS 2032</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1582,7 @@
         <f>Valuation!D16</f>
         <v/>
       </c>
-      <c r="D9" s="55">
+      <c r="D9" s="77">
         <f>Valuation!C21</f>
         <v/>
       </c>
@@ -2098,112 +2096,95 @@
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="O40" s="26" t="inlineStr">
-        <is>
-          <t>USE OF FUNDS (helper — chart data)</t>
-        </is>
-      </c>
-      <c r="P40" s="26" t="n"/>
-    </row>
-    <row r="41">
-      <c r="O41" s="26" t="inlineStr">
+    <row r="88">
+      <c r="B88" s="78" t="inlineStr">
+        <is>
+          <t>CHART DATA (calculated — do not edit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="26" t="inlineStr">
         <is>
           <t>App build</t>
         </is>
       </c>
-      <c r="P41" s="26" t="n">
+      <c r="C89" s="26" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="42">
-      <c r="O42" s="26" t="inlineStr">
+    <row r="90">
+      <c r="B90" s="26" t="inlineStr">
         <is>
           <t>Ops &amp; Team</t>
         </is>
       </c>
-      <c r="P42" s="26" t="n">
+      <c r="C90" s="26" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="43">
-      <c r="O43" s="26" t="inlineStr">
+    <row r="91">
+      <c r="B91" s="26" t="inlineStr">
         <is>
           <t>Market &amp; brand</t>
         </is>
       </c>
-      <c r="P43" s="26" t="n">
+      <c r="C91" s="26" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="44">
-      <c r="O44" s="26" t="inlineStr">
+    <row r="92">
+      <c r="B92" s="26" t="inlineStr">
         <is>
           <t>Simulators</t>
         </is>
       </c>
-      <c r="P44" s="26" t="n">
+      <c r="C92" s="26" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="45">
-      <c r="O45" s="26" t="inlineStr">
+    <row r="93">
+      <c r="B93" s="26" t="inlineStr">
         <is>
           <t>Pilot</t>
         </is>
       </c>
-      <c r="P45" s="26" t="n">
+      <c r="C93" s="26" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="46">
-      <c r="O46" s="26" t="n"/>
-      <c r="P46" s="26" t="n"/>
-    </row>
-    <row r="47">
-      <c r="O47" s="26" t="inlineStr">
-        <is>
-          <t>MILESTONES (helper — chart data)</t>
-        </is>
-      </c>
-      <c r="P47" s="26" t="n"/>
-    </row>
-    <row r="48">
-      <c r="O48" s="26" t="inlineStr">
+    <row r="95">
+      <c r="B95" s="26" t="inlineStr">
         <is>
           <t>This round</t>
         </is>
       </c>
-      <c r="P48" s="26">
+      <c r="C95" s="26">
         <f>Valuation!C10</f>
         <v/>
       </c>
     </row>
-    <row r="49">
-      <c r="O49" s="26" t="inlineStr">
+    <row r="96">
+      <c r="B96" s="26" t="inlineStr">
         <is>
           <t>Dec 2029</t>
         </is>
       </c>
-      <c r="P49" s="26">
+      <c r="C96" s="26">
         <f>Valuation!D10</f>
         <v/>
       </c>
     </row>
-    <row r="50">
-      <c r="O50" s="26" t="inlineStr">
+    <row r="97">
+      <c r="B97" s="26" t="inlineStr">
         <is>
           <t>2032</t>
         </is>
       </c>
-      <c r="P50" s="26">
+      <c r="C97" s="26">
         <f>Valuation!E10</f>
         <v/>
       </c>
-    </row>
-    <row r="51">
-      <c r="O51" s="26" t="n"/>
-      <c r="P51" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Pro forma headings given context on every sheet
Each sheet and dashboard table now says what it shows and how to read
it: Assumptions (blue cells restate the book; the site quotes this
sheet), Build (the 72-month engine every sheet reads from), Annual (net
streams add; memo lines are the insurer's view), Valuation (flat 3.0x
compressing from 3.69x; marks not returns), Dashboard tables (rows add /
trough inside the raise / multiple discipline) and the Insurance tier
ladder economics.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H812bzJCmkxEBTne82bnSQ
</commit_message>
<xml_diff>
--- a/GetLucky_Pro_Forma_v4.xlsx
+++ b/GetLucky_Pro_Forma_v4.xlsx
@@ -1597,6 +1597,11 @@
           <t>REVENUE BY STREAM (ZAR)</t>
         </is>
       </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Streams net of third-party shares — the rows add. Peer money in play is a KPI, never revenue.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="17" t="n"/>
@@ -1823,6 +1828,11 @@
           <t>PROFITABILITY &amp; CASH (ZAR)</t>
         </is>
       </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Costs budgeted line by line. The cumulative-cash trough is the peak drawdown — inside the R8m raise.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="17" t="n"/>
@@ -2016,6 +2026,11 @@
       <c r="B31" s="16" t="inlineStr">
         <is>
           <t>VALUATION &amp; THE INVESTOR</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>Flat 3.0× revenue at every forward milestone, compressing from the 3.69× this round implies.</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2247,7 @@
     <row r="3">
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Blue = change me. Black = calculated.</t>
+          <t>Every input in the book, in blue — change any blue cell and the whole workbook restates. The pitch site and dataroom quote this sheet at these values.</t>
         </is>
       </c>
     </row>
@@ -2800,9 +2815,9 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="38" t="inlineStr">
-        <is>
-          <t>Subscribers from ZERO. Milestone is month 36 (Dec 2029).</t>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>The 72-month engine: subscribers from zero (Jan 2027) → actives → money slips → jackpot entries and peer GMV, month by month. Every other sheet reads from here. Milestone is month 36 (Dec 2029).</t>
         </is>
       </c>
     </row>
@@ -8257,7 +8272,7 @@
     <row r="3">
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Calendar-year totals from the monthly build.</t>
+          <t>Calendar-year totals from the monthly build. Streams are net of third-party shares so the rows add; the memo lines show the insurer's view (gross entries, premium ceded, expected claims).</t>
         </is>
       </c>
     </row>
@@ -9139,6 +9154,11 @@
           <t>TIER LADDER</t>
         </is>
       </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Entry → insured prize, with the mix realised across 10,000 trailing entries. $17.00 weighted entry · $4.08 premium · $1.30 expected claim → 31.9% loss ratio, 2.51× breakeven.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="6" t="inlineStr">
@@ -9440,7 +9460,14 @@
     <row r="2">
       <c r="B2" s="27" t="inlineStr">
         <is>
-          <t>VALUATION</t>
+          <t>VALUATION &amp; INVESTOR RETURNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Milestones struck at a flat 3.0× revenue — the round implies 3.69×, so the rating compresses as the company scales. Returns shown on the full R8m for 15%; unrealised marks, not realised returns.</t>
         </is>
       </c>
     </row>

</xml_diff>